<commit_message>
Support full PI DataLink tag paths (\\SERVER\area.loop.PV)
- Excel template builds \\server\prefix+loop+suffix from Setup cells.
- Tuner derives the loop tag from full-path headers and guesses loop type
  from the instrument letters of the last segment.
- pi-check accepts a \\SERVER\tag path in the tag box.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HwFdZs7F7xgrizMmG418Sq
</commit_message>
<xml_diff>
--- a/pid-tuner/excel/PI_Tuner_Template.xlsx
+++ b/pid-tuner/excel/PI_Tuner_Template.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>แท็บ Setup: ใส่ชื่อ loop ในช่อง B4 (เช่น 3AC1102B) และตรวจว่า suffix .PV .SV .MV .MODE ตรงกับชื่อ tag ใน PI</t>
+          <t>แท็บ Setup: ตรวจ PI server (B4), area prefix (B5), ชื่อ loop (B6) และ suffix ให้ได้ชื่อ tag เต็มตรงกับที่ใช้ใน DataLink เช่น \\GCMPPISVR\3-CTA.2M.3AC1102B.MV</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Start time: คลิกเซลล์ Setup!B10 · End time: Setup!B11 · Time interval: Setup!B12 (หรือพิมพ์ *-2h, *, 1s ตรงๆ ก็ได้)</t>
+          <t>Start time: คลิกเซลล์ Setup!B12 · End time: Setup!B13 · Time interval: Setup!B14 (หรือพิมพ์ *-2h, *, 1s ตรงๆ ก็ได้)</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>เปิดไฟล์ แล้วแก้ชื่อ loop ที่ Setup!B4</t>
+          <t>เปิดไฟล์ แล้วแก้ชื่อ loop ที่ Setup!B6 (ถ้าเปลี่ยน area ให้แก้ B5 ด้วย)</t>
         </is>
       </c>
     </row>
@@ -692,6 +692,18 @@
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>ถ้า tag .SV หรือ .MODE ไม่มีใน PI (ช่องขึ้น error) ให้ค้นชื่อจริงด้วย PI DataLink → Search แล้วแก้ suffix ใน Setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>ไฟล์นี้ไม่มีสูตร PI DataLink มาให้ ต้องสร้างด้วยหน้าต่าง Sampled Data ตามข้อ 3–6 เพราะสูตรต้องสร้างบนเครื่องที่ต่อ PI ได้</t>
         </is>
@@ -708,11 +720,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -733,194 +745,228 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Loop tag</t>
+          <t>PI server</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>3AC1102B</t>
+          <t>GCMPPISVR</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ชื่อ loop ใน PI (ไม่ต้องใส่ .PV) เปลี่ยนช่องนี้ช่องเดียวเมื่อจะดู loop อื่น</t>
+          <t>ชื่อ PI Data Server (ส่วน \\GCMPPISVR\ ในชื่อ tag ของ DataLink)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PV suffix</t>
+          <t>Area prefix</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>.PV</t>
+          <t>3-CTA.2M.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ถ้าชื่อ tag ใน PI ต่างจากนี้ แก้ได้</t>
+          <t>ส่วนหน้าชื่อ tag ของพื้นที่นั้น (รวมจุดท้าย) ปกติไม่ต้องเปลี่ยนถ้าอยู่ area เดิม</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SV suffix</t>
+          <t>Loop tag</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>.SV</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
+          <t>3AC1102B</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>ชื่อ loop เปลี่ยนช่องนี้ช่องเดียวเมื่อจะดู loop อื่น</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MV suffix</t>
+          <t>PV suffix</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>.MV</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
+          <t>.PV</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>ถ้าชื่อ tag ใน PI ต่างจากนี้ แก้ได้</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MODE suffix</t>
+          <t>SV suffix</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>.MODE</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>ถ้าไม่มี tag MODE ใน PI ปล่อยไว้ได้ แอปยังใช้งานได้</t>
-        </is>
-      </c>
+          <t>.SV</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>MV suffix</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>.MV</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Start time</t>
+          <t>MODE suffix</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>*-2h</t>
+          <t>.MODE</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>PI time: *-2h = ย้อนหลัง 2 ชั่วโมง</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>End time</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>* = ตอนนี้</t>
+          <t>ถ้าไม่มี tag MODE ใน PI ปล่อยไว้ได้ แอปยังใช้งานได้</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Interval</t>
+          <t>Start time</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>1s</t>
+          <t>*-2h</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>flow/pressure 1s · temperature 5s · level 1–5s</t>
+          <t>PI time: *-2h = ย้อนหลัง 2 ชั่วโมง</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>End time</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>* = ตอนนี้</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Interval</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>1s</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>flow/pressure 1s · temperature 5s · level 1–5s</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>ชื่อ tag เต็ม (คำนวณให้)</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>PV</t>
-        </is>
-      </c>
-      <c r="B15" s="7">
-        <f>$B$4&amp;B5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>SV</t>
-        </is>
-      </c>
-      <c r="B16" s="7">
-        <f>$B$4&amp;B6</f>
-        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>MV</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="B17" s="7">
-        <f>$B$4&amp;B7</f>
+        <f>"\\"&amp;$B$4&amp;"\"&amp;$B$5&amp;$B$6&amp;B7</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="B18" s="7">
+        <f>"\\"&amp;$B$4&amp;"\"&amp;$B$5&amp;$B$6&amp;B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>MV</t>
+        </is>
+      </c>
+      <c r="B19" s="7">
+        <f>"\\"&amp;$B$4&amp;"\"&amp;$B$5&amp;$B$6&amp;B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>MODE</t>
         </is>
       </c>
-      <c r="B18" s="7">
-        <f>$B$4&amp;B8</f>
+      <c r="B20" s="7">
+        <f>"\\"&amp;$B$4&amp;"\"&amp;$B$5&amp;$B$6&amp;B10</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>สี:</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>ช่องที่แก้ได้</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>ค่าในช่องเหลืองตอนนี้เป็นตัวอย่าง (loop 3AC1102B ที่ใช้ทดสอบ)</t>
         </is>
@@ -941,10 +987,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -954,19 +1000,19 @@
         </is>
       </c>
       <c r="B1" s="9">
-        <f>Setup!$B$15</f>
-        <v/>
-      </c>
-      <c r="C1" s="9">
-        <f>Setup!$B$16</f>
-        <v/>
-      </c>
-      <c r="D1" s="9">
         <f>Setup!$B$17</f>
         <v/>
       </c>
+      <c r="C1" s="9">
+        <f>Setup!$B$18</f>
+        <v/>
+      </c>
+      <c r="D1" s="9">
+        <f>Setup!$B$19</f>
+        <v/>
+      </c>
       <c r="E1" s="9">
-        <f>Setup!$B$18</f>
+        <f>Setup!$B$20</f>
         <v/>
       </c>
       <c r="G1" s="5" t="inlineStr">

</xml_diff>